<commit_message>
update semantic seg 2.5 artifacts
</commit_message>
<xml_diff>
--- a/tests/perf_v2/perf_history/v2.5/semantic_segmentation/SEMANTIC_SEGMENTATION-aggregated.xlsx
+++ b/tests/perf_v2/perf_history/v2.5/semantic_segmentation/SEMANTIC_SEGMENTATION-aggregated.xlsx
@@ -588,52 +588,52 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>249.8699</v>
+        <v>264.3972</v>
       </c>
       <c r="C2" t="n">
-        <v>88.886</v>
+        <v>114.3917</v>
       </c>
       <c r="D2" t="n">
-        <v>28.8</v>
+        <v>30.6</v>
       </c>
       <c r="E2" t="n">
-        <v>10.7564</v>
+        <v>13.8311</v>
       </c>
       <c r="F2" t="n">
         <v>0.0442</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0003</v>
+        <v>0.0001</v>
       </c>
       <c r="H2" t="n">
-        <v>2.154</v>
+        <v>2.202</v>
       </c>
       <c r="I2" t="n">
-        <v>0.4724</v>
+        <v>0.5148</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7922</v>
+        <v>0.7925</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0023</v>
+        <v>0.0017</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7917999999999999</v>
+        <v>0.7919</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0021</v>
+        <v>0.0016</v>
       </c>
       <c r="N2" t="n">
-        <v>0.7911</v>
+        <v>0.7913</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0024</v>
+        <v>0.002</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0092</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0005</v>
+        <v>0.0002</v>
       </c>
       <c r="R2" t="n">
         <v>0.0861</v>
@@ -642,16 +642,16 @@
         <v>0.0009</v>
       </c>
       <c r="T2" t="n">
-        <v>0.0567</v>
+        <v>0.0574</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0009</v>
+        <v>0.0013</v>
       </c>
       <c r="V2" t="n">
-        <v>15.8301</v>
+        <v>16.0225</v>
       </c>
       <c r="W2" t="n">
-        <v>0.2404</v>
+        <v>0.3737</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -691,70 +691,70 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1449.2066</v>
+        <v>1483.4535</v>
       </c>
       <c r="C3" t="n">
-        <v>143.8108</v>
+        <v>131.0524</v>
       </c>
       <c r="D3" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E3" t="n">
-        <v>5.7879</v>
+        <v>5.1962</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1563</v>
+        <v>0.1572</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0004</v>
+        <v>0.0008</v>
       </c>
       <c r="H3" t="n">
-        <v>2.834</v>
+        <v>2.842</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0391</v>
+        <v>0.0409</v>
       </c>
       <c r="J3" t="n">
-        <v>0.7919</v>
+        <v>0.7923</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0029</v>
+        <v>0.0037</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7892</v>
+        <v>0.7899</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0031</v>
+        <v>0.0036</v>
       </c>
       <c r="N3" t="n">
-        <v>0.7842</v>
+        <v>0.7874</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0027</v>
+        <v>0.0032</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0141</v>
+        <v>0.0142</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0008</v>
+        <v>0.0009</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0499</v>
+        <v>0.0498</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0011</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0598</v>
+        <v>0.0606</v>
       </c>
       <c r="U3" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0015</v>
       </c>
       <c r="V3" t="n">
-        <v>16.6749</v>
+        <v>16.8978</v>
       </c>
       <c r="W3" t="n">
-        <v>0.1727</v>
+        <v>0.4053</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -794,70 +794,70 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1243.1934</v>
+        <v>1339.6073</v>
       </c>
       <c r="C4" t="n">
-        <v>186.2928</v>
+        <v>306.1477</v>
       </c>
       <c r="D4" t="n">
-        <v>57.6</v>
+        <v>62.4</v>
       </c>
       <c r="E4" t="n">
-        <v>8.848699999999999</v>
+        <v>14.2759</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1342</v>
+        <v>0.1337</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0009</v>
+        <v>0.0007</v>
       </c>
       <c r="H4" t="n">
-        <v>1.72</v>
+        <v>1.714</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0187</v>
+        <v>0.027</v>
       </c>
       <c r="J4" t="n">
-        <v>0.7638</v>
+        <v>0.7696</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0064</v>
+        <v>0.0124</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7621</v>
+        <v>0.7677</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0063</v>
+        <v>0.0125</v>
       </c>
       <c r="N4" t="n">
-        <v>0.7155</v>
+        <v>0.7328</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0135</v>
+        <v>0.0246</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0121</v>
+        <v>0.012</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0004</v>
+        <v>0.0005</v>
       </c>
       <c r="R4" t="n">
         <v>0.0529</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0009</v>
+        <v>0.0004</v>
       </c>
       <c r="T4" t="n">
-        <v>0.0703</v>
+        <v>0.0704</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0012</v>
+        <v>0.0022</v>
       </c>
       <c r="V4" t="n">
-        <v>19.6224</v>
+        <v>19.644</v>
       </c>
       <c r="W4" t="n">
-        <v>0.3223</v>
+        <v>0.608</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -897,70 +897,70 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2996.1506</v>
+        <v>2795.6988</v>
       </c>
       <c r="C5" t="n">
-        <v>411.8072</v>
+        <v>974.4056</v>
       </c>
       <c r="D5" t="n">
-        <v>58.8</v>
+        <v>54.8</v>
       </c>
       <c r="E5" t="n">
-        <v>8.167</v>
+        <v>19.5115</v>
       </c>
       <c r="F5" t="n">
-        <v>0.332</v>
+        <v>0.3322</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="H5" t="n">
-        <v>8.901999999999999</v>
+        <v>8.882</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0396</v>
+        <v>0.0259</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7952</v>
+        <v>0.7871</v>
       </c>
       <c r="K5" t="n">
-        <v>0.004</v>
+        <v>0.0229</v>
       </c>
       <c r="L5" t="n">
-        <v>0.792</v>
+        <v>0.7841</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0039</v>
+        <v>0.0228</v>
       </c>
       <c r="N5" t="n">
-        <v>0.433</v>
+        <v>0.6027</v>
       </c>
       <c r="O5" t="n">
-        <v>0.1814</v>
+        <v>0.0638</v>
       </c>
       <c r="P5" t="n">
-        <v>0.0217</v>
+        <v>0.0212</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0001</v>
       </c>
       <c r="R5" t="n">
-        <v>0.1216</v>
+        <v>0.1212</v>
       </c>
       <c r="S5" t="n">
         <v>0.0009</v>
       </c>
       <c r="T5" t="n">
-        <v>0.1317</v>
+        <v>0.1316</v>
       </c>
       <c r="U5" t="n">
-        <v>0.0011</v>
+        <v>0.0012</v>
       </c>
       <c r="V5" t="n">
-        <v>36.7305</v>
+        <v>36.7279</v>
       </c>
       <c r="W5" t="n">
-        <v>0.3067</v>
+        <v>0.3219</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -1000,70 +1000,70 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2361.209</v>
+        <v>1895.3292</v>
       </c>
       <c r="C6" t="n">
-        <v>376.0096</v>
+        <v>274.892</v>
       </c>
       <c r="D6" t="n">
-        <v>73.59999999999999</v>
+        <v>58.8</v>
       </c>
       <c r="E6" t="n">
-        <v>11.8659</v>
+        <v>8.642899999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2005</v>
+        <v>0.201</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
       <c r="H6" t="n">
-        <v>7.51</v>
+        <v>7.528</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0505</v>
+        <v>0.0585</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8250999999999999</v>
+        <v>0.8224</v>
       </c>
       <c r="K6" t="n">
-        <v>0.004</v>
+        <v>0.0051</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8228</v>
+        <v>0.8202</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0036</v>
+        <v>0.0052</v>
       </c>
       <c r="N6" t="n">
-        <v>0.8197</v>
+        <v>0.8159</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0052</v>
+        <v>0.0059</v>
       </c>
       <c r="P6" t="n">
-        <v>0.016</v>
+        <v>0.0163</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="R6" t="n">
-        <v>0.09180000000000001</v>
+        <v>0.0922</v>
       </c>
       <c r="S6" t="n">
-        <v>0.0013</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="T6" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.0738</v>
       </c>
       <c r="U6" t="n">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="V6" t="n">
-        <v>20.1952</v>
+        <v>20.5828</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1523</v>
+        <v>0.2904</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -1103,70 +1103,70 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1248.1917</v>
+        <v>1244.5198</v>
       </c>
       <c r="C7" t="n">
-        <v>253.4658</v>
+        <v>279.1601</v>
       </c>
       <c r="D7" t="n">
-        <v>60.6</v>
+        <v>60.8</v>
       </c>
       <c r="E7" t="n">
-        <v>12.341</v>
+        <v>14.1669</v>
       </c>
       <c r="F7" t="n">
         <v>0.1264</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0012</v>
       </c>
       <c r="H7" t="n">
-        <v>5.038</v>
+        <v>5.028</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0653</v>
+        <v>0.1397</v>
       </c>
       <c r="J7" t="n">
-        <v>0.8107</v>
+        <v>0.8096</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0039</v>
+        <v>0.0073</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8088</v>
+        <v>0.8076</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0042</v>
+        <v>0.0071</v>
       </c>
       <c r="N7" t="n">
-        <v>0.8064</v>
+        <v>0.8048</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0047</v>
+        <v>0.0075</v>
       </c>
       <c r="P7" t="n">
-        <v>0.0112</v>
+        <v>0.0114</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0002</v>
+        <v>0.0004</v>
       </c>
       <c r="R7" t="n">
-        <v>0.0587</v>
+        <v>0.0578</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0016</v>
+        <v>0.0011</v>
       </c>
       <c r="T7" t="n">
-        <v>0.0506</v>
+        <v>0.0491</v>
       </c>
       <c r="U7" t="n">
-        <v>0.0031</v>
+        <v>0.0005</v>
       </c>
       <c r="V7" t="n">
-        <v>14.1276</v>
+        <v>13.7027</v>
       </c>
       <c r="W7" t="n">
-        <v>0.8779</v>
+        <v>0.1519</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -1206,70 +1206,70 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1429.2097</v>
+        <v>1442.0677</v>
       </c>
       <c r="C8" t="n">
-        <v>106.1124</v>
+        <v>296.1351</v>
       </c>
       <c r="D8" t="n">
-        <v>77.59999999999999</v>
+        <v>78</v>
       </c>
       <c r="E8" t="n">
-        <v>5.7706</v>
+        <v>16.8819</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1143</v>
+        <v>0.1151</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0002</v>
+        <v>0.0014</v>
       </c>
       <c r="H8" t="n">
-        <v>3.806</v>
+        <v>3.724</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0956</v>
+        <v>0.08989999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8002</v>
+        <v>0.7996</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0027</v>
+        <v>0.0042</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7984</v>
+        <v>0.7978</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0027</v>
+        <v>0.0039</v>
       </c>
       <c r="N8" t="n">
-        <v>0.7963</v>
+        <v>0.7961</v>
       </c>
       <c r="O8" t="n">
-        <v>0.0035</v>
+        <v>0.0047</v>
       </c>
       <c r="P8" t="n">
         <v>0.009900000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.0003</v>
+        <v>0.0004</v>
       </c>
       <c r="R8" t="n">
-        <v>0.0452</v>
+        <v>0.0447</v>
       </c>
       <c r="S8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0009</v>
       </c>
       <c r="T8" t="n">
-        <v>0.047</v>
+        <v>0.0471</v>
       </c>
       <c r="U8" t="n">
         <v>0.0009</v>
       </c>
       <c r="V8" t="n">
-        <v>13.1105</v>
+        <v>13.1534</v>
       </c>
       <c r="W8" t="n">
-        <v>0.2492</v>
+        <v>0.254</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
@@ -1470,70 +1470,70 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24.6398</v>
+        <v>90.389</v>
       </c>
       <c r="C2" t="n">
-        <v>9.434900000000001</v>
+        <v>14.5994</v>
       </c>
       <c r="D2" t="n">
-        <v>12.4</v>
+        <v>51.2</v>
       </c>
       <c r="E2" t="n">
-        <v>5.3666</v>
+        <v>8.8994</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0543</v>
+        <v>0.0549</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0002</v>
+        <v>0.0004</v>
       </c>
       <c r="H2" t="n">
-        <v>1.312</v>
+        <v>1.676</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1381</v>
+        <v>0.1205</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5758</v>
+        <v>0.6468</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0315</v>
+        <v>0.0022</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5741000000000001</v>
+        <v>0.6443</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0313</v>
+        <v>0.0021</v>
       </c>
       <c r="N2" t="n">
-        <v>0.5756</v>
+        <v>0.6467000000000001</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0343</v>
+        <v>0.002</v>
       </c>
       <c r="P2" t="n">
         <v>0.0281</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0007</v>
+        <v>0.0008</v>
       </c>
       <c r="R2" t="n">
-        <v>0.2342</v>
+        <v>0.2373</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0022</v>
+        <v>0.0026</v>
       </c>
       <c r="T2" t="n">
-        <v>0.2323</v>
+        <v>0.2305</v>
       </c>
       <c r="U2" t="n">
         <v>0.0036</v>
       </c>
       <c r="V2" t="n">
-        <v>11.6158</v>
+        <v>11.5252</v>
       </c>
       <c r="W2" t="n">
-        <v>0.1776</v>
+        <v>0.179</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -1573,70 +1573,70 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>114.1059</v>
+        <v>277.8922</v>
       </c>
       <c r="C3" t="n">
-        <v>12.1216</v>
+        <v>102.6702</v>
       </c>
       <c r="D3" t="n">
-        <v>28.6</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>3.2863</v>
+        <v>27.2819</v>
       </c>
       <c r="F3" t="n">
-        <v>0.161</v>
+        <v>0.1617</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0005</v>
+        <v>0.0008</v>
       </c>
       <c r="H3" t="n">
-        <v>2.906</v>
+        <v>2.908</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0207</v>
+        <v>0.0217</v>
       </c>
       <c r="J3" t="n">
-        <v>0.4226</v>
+        <v>0.4632</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0169</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="L3" t="n">
-        <v>0.4217</v>
+        <v>0.4626</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0172</v>
+        <v>0.0098</v>
       </c>
       <c r="N3" t="n">
-        <v>0.4172</v>
+        <v>0.4553</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0182</v>
+        <v>0.0131</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0406</v>
+        <v>0.0379</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0034</v>
+        <v>0.0027</v>
       </c>
       <c r="R3" t="n">
-        <v>0.2456</v>
+        <v>0.2379</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0094</v>
+        <v>0.0025</v>
       </c>
       <c r="T3" t="n">
-        <v>0.3028</v>
+        <v>0.3108</v>
       </c>
       <c r="U3" t="n">
-        <v>0.0132</v>
+        <v>0.0124</v>
       </c>
       <c r="V3" t="n">
-        <v>15.1403</v>
+        <v>15.5382</v>
       </c>
       <c r="W3" t="n">
-        <v>0.6611</v>
+        <v>0.6176</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -1676,70 +1676,70 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>105.5346</v>
+        <v>258.1688</v>
       </c>
       <c r="C4" t="n">
-        <v>17.3115</v>
+        <v>41.7336</v>
       </c>
       <c r="D4" t="n">
-        <v>31</v>
+        <v>78.8</v>
       </c>
       <c r="E4" t="n">
-        <v>5.1962</v>
+        <v>13.0077</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1345</v>
+        <v>0.1332</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0015</v>
+        <v>0.0002</v>
       </c>
       <c r="H4" t="n">
-        <v>1.52</v>
+        <v>1.532</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0951</v>
+        <v>0.123</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3992</v>
+        <v>0.4498</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0219</v>
+        <v>0.0102</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3987</v>
+        <v>0.4489</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0218</v>
+        <v>0.0101</v>
       </c>
       <c r="N4" t="n">
-        <v>0.3433</v>
+        <v>0.391</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0441</v>
+        <v>0.0246</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0319</v>
+        <v>0.0332</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0009</v>
+        <v>0.0024</v>
       </c>
       <c r="R4" t="n">
-        <v>0.4001</v>
+        <v>0.4012</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0029</v>
+        <v>0.0044</v>
       </c>
       <c r="T4" t="n">
-        <v>0.4711</v>
+        <v>0.4845</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0067</v>
+        <v>0.0126</v>
       </c>
       <c r="V4" t="n">
-        <v>23.5566</v>
+        <v>24.2273</v>
       </c>
       <c r="W4" t="n">
-        <v>0.3367</v>
+        <v>0.6294</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -1779,70 +1779,70 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>159.4236</v>
+        <v>698.3392</v>
       </c>
       <c r="C5" t="n">
-        <v>62.7364</v>
+        <v>28.6936</v>
       </c>
       <c r="D5" t="n">
-        <v>20.8</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>8.642899999999999</v>
+        <v>3.9115</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3313</v>
+        <v>0.3316</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0017</v>
+        <v>0.0008</v>
       </c>
       <c r="H5" t="n">
-        <v>8.914</v>
+        <v>8.9</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0796</v>
+        <v>0.0224</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3572</v>
+        <v>0.4931</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0629</v>
+        <v>0.0083</v>
       </c>
       <c r="L5" t="n">
-        <v>0.357</v>
+        <v>0.4924</v>
       </c>
       <c r="M5" t="n">
-        <v>0.06270000000000001</v>
+        <v>0.0081</v>
       </c>
       <c r="N5" t="n">
-        <v>0.2548</v>
+        <v>0.2218</v>
       </c>
       <c r="O5" t="n">
-        <v>0.0464</v>
+        <v>0.0437</v>
       </c>
       <c r="P5" t="n">
-        <v>0.0562</v>
+        <v>0.0586</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.0033</v>
+        <v>0.003</v>
       </c>
       <c r="R5" t="n">
-        <v>0.3426</v>
+        <v>0.3464</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0071</v>
+        <v>0.0083</v>
       </c>
       <c r="T5" t="n">
-        <v>0.4856</v>
+        <v>0.486</v>
       </c>
       <c r="U5" t="n">
-        <v>0.0028</v>
+        <v>0.0058</v>
       </c>
       <c r="V5" t="n">
-        <v>24.2822</v>
+        <v>24.3</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1381</v>
+        <v>0.2894</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -1882,70 +1882,70 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>139.2863</v>
+        <v>708.6759</v>
       </c>
       <c r="C6" t="n">
-        <v>42.8366</v>
+        <v>217.883</v>
       </c>
       <c r="D6" t="n">
-        <v>26.8</v>
+        <v>143.6</v>
       </c>
       <c r="E6" t="n">
-        <v>8.642899999999999</v>
+        <v>44.7694</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2053</v>
+        <v>0.2054</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0004</v>
+        <v>0.0007</v>
       </c>
       <c r="H6" t="n">
-        <v>7.672</v>
+        <v>7.808</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0939</v>
+        <v>0.1018</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4192</v>
+        <v>0.6282</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0781</v>
+        <v>0.0629</v>
       </c>
       <c r="L6" t="n">
-        <v>0.4186</v>
+        <v>0.626</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0781</v>
+        <v>0.0623</v>
       </c>
       <c r="N6" t="n">
-        <v>0.3585</v>
+        <v>0.6141</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0505</v>
+        <v>0.0619</v>
       </c>
       <c r="P6" t="n">
-        <v>0.0474</v>
+        <v>0.0477</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.0031</v>
+        <v>0.0029</v>
       </c>
       <c r="R6" t="n">
-        <v>0.2666</v>
+        <v>0.2737</v>
       </c>
       <c r="S6" t="n">
-        <v>0.0123</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="T6" t="n">
-        <v>0.2988</v>
+        <v>0.3034</v>
       </c>
       <c r="U6" t="n">
         <v>0.0045</v>
       </c>
       <c r="V6" t="n">
-        <v>14.9412</v>
+        <v>15.1677</v>
       </c>
       <c r="W6" t="n">
-        <v>0.2246</v>
+        <v>0.2245</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -1985,70 +1985,70 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>120.2489</v>
+        <v>379.9241</v>
       </c>
       <c r="C7" t="n">
-        <v>47.1057</v>
+        <v>46.5829</v>
       </c>
       <c r="D7" t="n">
-        <v>36.4</v>
+        <v>119</v>
       </c>
       <c r="E7" t="n">
-        <v>14.758</v>
+        <v>15</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1239</v>
+        <v>0.1245</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0002</v>
+        <v>0.0005</v>
       </c>
       <c r="H7" t="n">
-        <v>4.62</v>
+        <v>4.77</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1037</v>
+        <v>0.0274</v>
       </c>
       <c r="J7" t="n">
-        <v>0.3826</v>
+        <v>0.5265</v>
       </c>
       <c r="K7" t="n">
-        <v>0.09909999999999999</v>
+        <v>0.0048</v>
       </c>
       <c r="L7" t="n">
-        <v>0.3821</v>
+        <v>0.5253</v>
       </c>
       <c r="M7" t="n">
-        <v>0.09909999999999999</v>
+        <v>0.0049</v>
       </c>
       <c r="N7" t="n">
-        <v>0.3798</v>
+        <v>0.5201</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0992</v>
+        <v>0.0073</v>
       </c>
       <c r="P7" t="n">
-        <v>0.0314</v>
+        <v>0.033</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.003</v>
       </c>
       <c r="R7" t="n">
-        <v>0.2246</v>
+        <v>0.2208</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0072</v>
+        <v>0.0027</v>
       </c>
       <c r="T7" t="n">
-        <v>0.2394</v>
+        <v>0.244</v>
       </c>
       <c r="U7" t="n">
-        <v>0.0064</v>
+        <v>0.0065</v>
       </c>
       <c r="V7" t="n">
-        <v>11.9687</v>
+        <v>12.1982</v>
       </c>
       <c r="W7" t="n">
-        <v>0.3201</v>
+        <v>0.327</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -2088,70 +2088,70 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>161.4605</v>
+        <v>353.1456</v>
       </c>
       <c r="C8" t="n">
-        <v>44.8127</v>
+        <v>61.2972</v>
       </c>
       <c r="D8" t="n">
-        <v>55.6</v>
+        <v>124.4</v>
       </c>
       <c r="E8" t="n">
-        <v>16.0717</v>
+        <v>22.1878</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1126</v>
+        <v>0.1127</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0009</v>
+        <v>0.0004</v>
       </c>
       <c r="H8" t="n">
-        <v>3.464</v>
+        <v>3.494</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0241</v>
+        <v>0.0358</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3997</v>
+        <v>0.4946</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0641</v>
+        <v>0.0134</v>
       </c>
       <c r="L8" t="n">
-        <v>0.3995</v>
+        <v>0.4939</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0641</v>
+        <v>0.0135</v>
       </c>
       <c r="N8" t="n">
-        <v>0.3828</v>
+        <v>0.4824</v>
       </c>
       <c r="O8" t="n">
-        <v>0.0536</v>
+        <v>0.0185</v>
       </c>
       <c r="P8" t="n">
-        <v>0.0283</v>
+        <v>0.0279</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0003</v>
       </c>
       <c r="R8" t="n">
-        <v>0.2192</v>
+        <v>0.2157</v>
       </c>
       <c r="S8" t="n">
         <v>0.0022</v>
       </c>
       <c r="T8" t="n">
-        <v>0.2494</v>
+        <v>0.2437</v>
       </c>
       <c r="U8" t="n">
-        <v>0.0044</v>
+        <v>0.0075</v>
       </c>
       <c r="V8" t="n">
-        <v>12.4684</v>
+        <v>12.1835</v>
       </c>
       <c r="W8" t="n">
-        <v>0.2214</v>
+        <v>0.3753</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
@@ -2352,10 +2352,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>177.0713</v>
+        <v>176.0062</v>
       </c>
       <c r="C2" t="n">
-        <v>40.2343</v>
+        <v>38.8639</v>
       </c>
       <c r="D2" t="n">
         <v>20.8</v>
@@ -2364,58 +2364,58 @@
         <v>4.9699</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0576</v>
+        <v>0.0577</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0002</v>
+        <v>0.0003</v>
       </c>
       <c r="H2" t="n">
-        <v>3.062</v>
+        <v>2.648</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2199</v>
+        <v>0.2994</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8665</v>
+        <v>0.8661</v>
       </c>
       <c r="K2" t="n">
         <v>0.0045</v>
       </c>
       <c r="L2" t="n">
-        <v>0.8649</v>
+        <v>0.8646</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0048</v>
+        <v>0.0047</v>
       </c>
       <c r="N2" t="n">
-        <v>0.8645</v>
+        <v>0.8643999999999999</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0056</v>
+        <v>0.0055</v>
       </c>
       <c r="P2" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0104</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0001</v>
+        <v>0.002</v>
       </c>
       <c r="R2" t="n">
-        <v>0.1163</v>
+        <v>0.1181</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0014</v>
+        <v>0.0041</v>
       </c>
       <c r="T2" t="n">
-        <v>0.0919</v>
+        <v>0.0948</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0017</v>
+        <v>0.0032</v>
       </c>
       <c r="V2" t="n">
-        <v>27.5844</v>
+        <v>28.4441</v>
       </c>
       <c r="W2" t="n">
-        <v>0.4961</v>
+        <v>0.958</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -2455,70 +2455,70 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1119.2089</v>
+        <v>1123.7968</v>
       </c>
       <c r="C3" t="n">
-        <v>242.9613</v>
+        <v>247.5455</v>
       </c>
       <c r="D3" t="n">
-        <v>62.6</v>
+        <v>63</v>
       </c>
       <c r="E3" t="n">
-        <v>14.0641</v>
+        <v>14.089</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1597</v>
+        <v>0.1592</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0014</v>
+        <v>0.0002</v>
       </c>
       <c r="H3" t="n">
-        <v>3.562</v>
+        <v>3.508</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1047</v>
+        <v>0.07920000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>0.4549</v>
+        <v>0.4289</v>
       </c>
       <c r="K3" t="n">
-        <v>0.021</v>
+        <v>0.0165</v>
       </c>
       <c r="L3" t="n">
-        <v>0.4519</v>
+        <v>0.4261</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0216</v>
+        <v>0.0167</v>
       </c>
       <c r="N3" t="n">
-        <v>0.4236</v>
+        <v>0.3819</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0192</v>
+        <v>0.0308</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0143</v>
+        <v>0.0147</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0005</v>
+        <v>0.0002</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0912</v>
+        <v>0.091</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0016</v>
+        <v>0.0012</v>
       </c>
       <c r="T3" t="n">
-        <v>0.099</v>
+        <v>0.0987</v>
       </c>
       <c r="U3" t="n">
-        <v>0.0016</v>
+        <v>0.0019</v>
       </c>
       <c r="V3" t="n">
-        <v>29.6972</v>
+        <v>29.6036</v>
       </c>
       <c r="W3" t="n">
-        <v>0.4701</v>
+        <v>0.5839</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -2558,70 +2558,70 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1062.0106</v>
+        <v>1044.2531</v>
       </c>
       <c r="C4" t="n">
-        <v>228.0649</v>
+        <v>110.7656</v>
       </c>
       <c r="D4" t="n">
-        <v>68.2</v>
+        <v>67</v>
       </c>
       <c r="E4" t="n">
-        <v>14.9566</v>
+        <v>7.4833</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1374</v>
+        <v>0.1376</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0012</v>
       </c>
       <c r="H4" t="n">
-        <v>2.43</v>
+        <v>2.454</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1068</v>
+        <v>0.1031</v>
       </c>
       <c r="J4" t="n">
-        <v>0.421</v>
+        <v>0.4375</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0461</v>
+        <v>0.0169</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4206</v>
+        <v>0.4359</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0462</v>
+        <v>0.0156</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1566</v>
+        <v>0.2125</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0689</v>
+        <v>0.0171</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0128</v>
+        <v>0.0127</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0005</v>
+        <v>0.0008</v>
       </c>
       <c r="R4" t="n">
-        <v>0.1501</v>
+        <v>0.149</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0022</v>
       </c>
       <c r="T4" t="n">
-        <v>0.1654</v>
+        <v>0.1661</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0045</v>
+        <v>0.0011</v>
       </c>
       <c r="V4" t="n">
-        <v>49.6088</v>
+        <v>49.8431</v>
       </c>
       <c r="W4" t="n">
-        <v>1.3431</v>
+        <v>0.3296</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -2661,70 +2661,70 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2320.8871</v>
+        <v>2115.6203</v>
       </c>
       <c r="C5" t="n">
-        <v>269.3897</v>
+        <v>1108.5954</v>
       </c>
       <c r="D5" t="n">
-        <v>67.8</v>
+        <v>61.6</v>
       </c>
       <c r="E5" t="n">
-        <v>8.012499999999999</v>
+        <v>32.807</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3339</v>
+        <v>0.3343</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0004</v>
+        <v>0.001</v>
       </c>
       <c r="H5" t="n">
-        <v>9.458</v>
+        <v>9.484</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0239</v>
+        <v>0.0378</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3777</v>
+        <v>0.3052</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0205</v>
+        <v>0.0955</v>
       </c>
       <c r="L5" t="n">
-        <v>0.3778</v>
+        <v>0.3051</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0212</v>
+        <v>0.0959</v>
       </c>
       <c r="N5" t="n">
-        <v>0.0762</v>
+        <v>0.0589</v>
       </c>
       <c r="O5" t="n">
-        <v>0.0238</v>
+        <v>0.0114</v>
       </c>
       <c r="P5" t="n">
-        <v>0.0221</v>
+        <v>0.0215</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.0003</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="R5" t="n">
-        <v>0.1571</v>
+        <v>0.1562</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0017</v>
+        <v>0.0018</v>
       </c>
       <c r="T5" t="n">
-        <v>0.168</v>
+        <v>0.1696</v>
       </c>
       <c r="U5" t="n">
-        <v>0.0014</v>
+        <v>0.0016</v>
       </c>
       <c r="V5" t="n">
-        <v>50.3969</v>
+        <v>50.8927</v>
       </c>
       <c r="W5" t="n">
-        <v>0.4226</v>
+        <v>0.4849</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -2764,70 +2764,70 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>664.6531</v>
+        <v>794.8181</v>
       </c>
       <c r="C6" t="n">
-        <v>133.4001</v>
+        <v>207.8824</v>
       </c>
       <c r="D6" t="n">
-        <v>28.8</v>
+        <v>34.8</v>
       </c>
       <c r="E6" t="n">
-        <v>6.0992</v>
+        <v>9.5237</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2049</v>
+        <v>0.2043</v>
       </c>
       <c r="G6" t="n">
         <v>0.0002</v>
       </c>
       <c r="H6" t="n">
-        <v>8.316000000000001</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>0.07920000000000001</v>
+        <v>0.1173</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8297</v>
+        <v>0.8326</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0073</v>
+        <v>0.0075</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8274</v>
+        <v>0.8318</v>
       </c>
       <c r="M6" t="n">
         <v>0.0068</v>
       </c>
       <c r="N6" t="n">
-        <v>0.8192</v>
+        <v>0.8209</v>
       </c>
       <c r="O6" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0207</v>
       </c>
       <c r="P6" t="n">
-        <v>0.0162</v>
+        <v>0.0164</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.0004</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="R6" t="n">
         <v>0.1261</v>
       </c>
       <c r="S6" t="n">
-        <v>0.001</v>
+        <v>0.0001</v>
       </c>
       <c r="T6" t="n">
-        <v>0.1103</v>
+        <v>0.1123</v>
       </c>
       <c r="U6" t="n">
-        <v>0.0023</v>
+        <v>0.0019</v>
       </c>
       <c r="V6" t="n">
-        <v>33.0923</v>
+        <v>33.6761</v>
       </c>
       <c r="W6" t="n">
-        <v>0.6991000000000001</v>
+        <v>0.579</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -2867,70 +2867,70 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>681.3765</v>
+        <v>785.2026</v>
       </c>
       <c r="C7" t="n">
-        <v>96.3352</v>
+        <v>210.6798</v>
       </c>
       <c r="D7" t="n">
-        <v>45.4</v>
+        <v>53</v>
       </c>
       <c r="E7" t="n">
-        <v>6.6933</v>
+        <v>14.5945</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1293</v>
+        <v>0.1285</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0011</v>
+        <v>0.0008</v>
       </c>
       <c r="H7" t="n">
-        <v>6.048</v>
+        <v>6.054</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1966</v>
+        <v>0.1474</v>
       </c>
       <c r="J7" t="n">
-        <v>0.8053</v>
+        <v>0.8102</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0048</v>
+        <v>0.0101</v>
       </c>
       <c r="L7" t="n">
-        <v>0.803</v>
+        <v>0.8078</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0055</v>
+        <v>0.0102</v>
       </c>
       <c r="N7" t="n">
-        <v>0.7992</v>
+        <v>0.8004</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0042</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="P7" t="n">
-        <v>0.0118</v>
+        <v>0.012</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0002</v>
+        <v>0.0004</v>
       </c>
       <c r="R7" t="n">
-        <v>0.0954</v>
+        <v>0.09760000000000001</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0008</v>
+        <v>0.0016</v>
       </c>
       <c r="T7" t="n">
-        <v>0.0868</v>
+        <v>0.0892</v>
       </c>
       <c r="U7" t="n">
-        <v>0.0031</v>
+        <v>0.0015</v>
       </c>
       <c r="V7" t="n">
-        <v>26.0271</v>
+        <v>26.7598</v>
       </c>
       <c r="W7" t="n">
-        <v>0.9367</v>
+        <v>0.4603</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -2970,70 +2970,70 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>745.4105</v>
+        <v>652.972</v>
       </c>
       <c r="C8" t="n">
-        <v>121.3614</v>
+        <v>148.5232</v>
       </c>
       <c r="D8" t="n">
-        <v>55</v>
+        <v>48.4</v>
       </c>
       <c r="E8" t="n">
-        <v>9.055400000000001</v>
+        <v>11.6103</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1185</v>
+        <v>0.1173</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0018</v>
+        <v>0.0009</v>
       </c>
       <c r="H8" t="n">
-        <v>4.562</v>
+        <v>4.644</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0526</v>
+        <v>0.0844</v>
       </c>
       <c r="J8" t="n">
-        <v>0.7783</v>
+        <v>0.7747000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0107</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7763</v>
+        <v>0.7725</v>
       </c>
       <c r="M8" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0104</v>
       </c>
       <c r="N8" t="n">
-        <v>0.7734</v>
+        <v>0.7691</v>
       </c>
       <c r="O8" t="n">
-        <v>0.01</v>
+        <v>0.0122</v>
       </c>
       <c r="P8" t="n">
         <v>0.0105</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.0007</v>
+        <v>0.0004</v>
       </c>
       <c r="R8" t="n">
-        <v>0.0861</v>
+        <v>0.0852</v>
       </c>
       <c r="S8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.001</v>
       </c>
       <c r="T8" t="n">
-        <v>0.0873</v>
+        <v>0.0868</v>
       </c>
       <c r="U8" t="n">
-        <v>0.0021</v>
+        <v>0.0022</v>
       </c>
       <c r="V8" t="n">
-        <v>26.1769</v>
+        <v>26.042</v>
       </c>
       <c r="W8" t="n">
-        <v>0.6311</v>
+        <v>0.6642</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
@@ -3234,70 +3234,70 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24.4761</v>
+        <v>65.6294</v>
       </c>
       <c r="C2" t="n">
-        <v>6.4351</v>
+        <v>13.0756</v>
       </c>
       <c r="D2" t="n">
-        <v>24.4</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>6.9498</v>
+        <v>15.1261</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0561</v>
+        <v>0.0568</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0005</v>
+        <v>0.0002</v>
       </c>
       <c r="H2" t="n">
-        <v>1.202</v>
+        <v>1.17</v>
       </c>
       <c r="I2" t="n">
-        <v>0.08840000000000001</v>
+        <v>0.0071</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5357</v>
+        <v>0.5611</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0106</v>
+        <v>0.0068</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5357</v>
+        <v>0.5606</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0107</v>
+        <v>0.0068</v>
       </c>
       <c r="N2" t="n">
-        <v>0.5346</v>
+        <v>0.5606</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0106</v>
+        <v>0.0061</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0406</v>
+        <v>0.0413</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.001</v>
+        <v>0.0017</v>
       </c>
       <c r="R2" t="n">
-        <v>0.2932</v>
+        <v>0.2836</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0042</v>
+        <v>0.0019</v>
       </c>
       <c r="T2" t="n">
-        <v>0.3101</v>
+        <v>0.2991</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0074</v>
+        <v>0.0127</v>
       </c>
       <c r="V2" t="n">
-        <v>9.3024</v>
+        <v>8.9732</v>
       </c>
       <c r="W2" t="n">
-        <v>0.2216</v>
+        <v>0.3824</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -3337,70 +3337,70 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>74.7328</v>
+        <v>207.9008</v>
       </c>
       <c r="C3" t="n">
-        <v>31.104</v>
+        <v>33.0642</v>
       </c>
       <c r="D3" t="n">
-        <v>44.8</v>
+        <v>131</v>
       </c>
       <c r="E3" t="n">
-        <v>19.6774</v>
+        <v>21.3542</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1517</v>
+        <v>0.1504</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0009</v>
+        <v>0.0012</v>
       </c>
       <c r="H3" t="n">
-        <v>3.06</v>
+        <v>3.03</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>0.0274</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2986</v>
+        <v>0.449</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0982</v>
+        <v>0.013</v>
       </c>
       <c r="L3" t="n">
-        <v>0.2982</v>
+        <v>0.4486</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0975</v>
+        <v>0.0128</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2923</v>
+        <v>0.443</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0956</v>
+        <v>0.0159</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0569</v>
+        <v>0.0578</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0042</v>
+        <v>0.0048</v>
       </c>
       <c r="R3" t="n">
-        <v>0.3122</v>
+        <v>0.313</v>
       </c>
       <c r="S3" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.0115</v>
       </c>
       <c r="T3" t="n">
-        <v>0.3927</v>
+        <v>0.3953</v>
       </c>
       <c r="U3" t="n">
-        <v>0.0153</v>
+        <v>0.0208</v>
       </c>
       <c r="V3" t="n">
-        <v>11.7802</v>
+        <v>11.8581</v>
       </c>
       <c r="W3" t="n">
-        <v>0.4582</v>
+        <v>0.6237</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -3440,70 +3440,70 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54.3158</v>
+        <v>204.2748</v>
       </c>
       <c r="C4" t="n">
-        <v>5.9872</v>
+        <v>45.0779</v>
       </c>
       <c r="D4" t="n">
-        <v>37.6</v>
+        <v>150.2</v>
       </c>
       <c r="E4" t="n">
-        <v>4.5607</v>
+        <v>34.1057</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1239</v>
+        <v>0.1234</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0019</v>
+        <v>0.0009</v>
       </c>
       <c r="H4" t="n">
-        <v>1.442</v>
+        <v>1.528</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0045</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>0.2439</v>
+        <v>0.4226</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0194</v>
+        <v>0.0145</v>
       </c>
       <c r="L4" t="n">
-        <v>0.2439</v>
+        <v>0.4221</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0194</v>
+        <v>0.0145</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1789</v>
+        <v>0.3096</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0464</v>
+        <v>0.0466</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0489</v>
+        <v>0.054</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0016</v>
+        <v>0.0053</v>
       </c>
       <c r="R4" t="n">
-        <v>0.4523</v>
+        <v>0.4481</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0078</v>
+        <v>0.0062</v>
       </c>
       <c r="T4" t="n">
-        <v>0.5653</v>
+        <v>0.5735</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0199</v>
+        <v>0.0174</v>
       </c>
       <c r="V4" t="n">
-        <v>16.9577</v>
+        <v>17.2036</v>
       </c>
       <c r="W4" t="n">
-        <v>0.5984</v>
+        <v>0.5232</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -3543,70 +3543,70 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>136.0986</v>
+        <v>472.0184</v>
       </c>
       <c r="C5" t="n">
-        <v>42.4121</v>
+        <v>75.9178</v>
       </c>
       <c r="D5" t="n">
-        <v>44.8</v>
+        <v>162.2</v>
       </c>
       <c r="E5" t="n">
-        <v>14.5327</v>
+        <v>26.7432</v>
       </c>
       <c r="F5" t="n">
-        <v>0.332</v>
+        <v>0.3304</v>
       </c>
       <c r="G5" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="H5" t="n">
+        <v>8.978</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.0963</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.436</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.0381</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.4355</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.0382</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.1381</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.0822</v>
+      </c>
+      <c r="Q5" t="n">
         <v>0.0031</v>
       </c>
-      <c r="H5" t="n">
-        <v>8.917999999999999</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.0179</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.2639</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.0595</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.2635</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.0593</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.1142</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.0387</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.09089999999999999</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.0013</v>
-      </c>
       <c r="R5" t="n">
-        <v>0.4374</v>
+        <v>0.4408</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0113</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="T5" t="n">
-        <v>0.7069</v>
+        <v>0.7027</v>
       </c>
       <c r="U5" t="n">
-        <v>0.0271</v>
+        <v>0.0073</v>
       </c>
       <c r="V5" t="n">
-        <v>21.2056</v>
+        <v>21.0808</v>
       </c>
       <c r="W5" t="n">
-        <v>0.8121</v>
+        <v>0.2181</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -3646,70 +3646,70 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>135.6359</v>
+        <v>389.3589</v>
       </c>
       <c r="C6" t="n">
-        <v>35.2028</v>
+        <v>56.7246</v>
       </c>
       <c r="D6" t="n">
-        <v>62.4</v>
+        <v>186.2</v>
       </c>
       <c r="E6" t="n">
-        <v>16.6373</v>
+        <v>28.6217</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1987</v>
+        <v>0.1992</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0003</v>
+        <v>0.0004</v>
       </c>
       <c r="H6" t="n">
-        <v>7.772</v>
+        <v>7.77</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0045</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.3039</v>
+        <v>0.501</v>
       </c>
       <c r="K6" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.0209</v>
       </c>
       <c r="L6" t="n">
-        <v>0.3037</v>
+        <v>0.5004</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0931</v>
+        <v>0.0209</v>
       </c>
       <c r="N6" t="n">
-        <v>0.2856</v>
+        <v>0.4851</v>
       </c>
       <c r="O6" t="n">
-        <v>0.099</v>
+        <v>0.0354</v>
       </c>
       <c r="P6" t="n">
-        <v>0.0693</v>
+        <v>0.07240000000000001</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.0053</v>
+        <v>0.0057</v>
       </c>
       <c r="R6" t="n">
-        <v>0.3488</v>
+        <v>0.3406</v>
       </c>
       <c r="S6" t="n">
-        <v>0.0078</v>
+        <v>0.0146</v>
       </c>
       <c r="T6" t="n">
-        <v>0.406</v>
+        <v>0.4032</v>
       </c>
       <c r="U6" t="n">
-        <v>0.0141</v>
+        <v>0.0046</v>
       </c>
       <c r="V6" t="n">
-        <v>12.1801</v>
+        <v>12.0954</v>
       </c>
       <c r="W6" t="n">
-        <v>0.4224</v>
+        <v>0.1393</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -3749,70 +3749,70 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>64.33280000000001</v>
+        <v>278.9737</v>
       </c>
       <c r="C7" t="n">
-        <v>17.2109</v>
+        <v>2.0969</v>
       </c>
       <c r="D7" t="n">
-        <v>43.2</v>
+        <v>199</v>
       </c>
       <c r="E7" t="n">
-        <v>12.4579</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1194</v>
+        <v>0.1197</v>
       </c>
       <c r="G7" t="n">
         <v>0.0004</v>
       </c>
       <c r="H7" t="n">
-        <v>4.664</v>
+        <v>4.668</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0055</v>
+        <v>0.0045</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1567</v>
+        <v>0.4616</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0257</v>
+        <v>0.0058</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1567</v>
+        <v>0.461</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0258</v>
+        <v>0.0057</v>
       </c>
       <c r="N7" t="n">
-        <v>0.1571</v>
+        <v>0.4593</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0254</v>
+        <v>0.0053</v>
       </c>
       <c r="P7" t="n">
-        <v>0.0505</v>
+        <v>0.0485</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0051</v>
+        <v>0.0008</v>
       </c>
       <c r="R7" t="n">
-        <v>0.2765</v>
+        <v>0.2846</v>
       </c>
       <c r="S7" t="n">
-        <v>0.01</v>
+        <v>0.0049</v>
       </c>
       <c r="T7" t="n">
-        <v>0.3159</v>
+        <v>0.3157</v>
       </c>
       <c r="U7" t="n">
-        <v>0.012</v>
+        <v>0.007</v>
       </c>
       <c r="V7" t="n">
-        <v>9.478199999999999</v>
+        <v>9.471299999999999</v>
       </c>
       <c r="W7" t="n">
-        <v>0.3588</v>
+        <v>0.2108</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -3852,70 +3852,70 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>48.8456</v>
+        <v>243.739</v>
       </c>
       <c r="C8" t="n">
-        <v>26.0556</v>
+        <v>0.7625</v>
       </c>
       <c r="D8" t="n">
-        <v>37.6</v>
+        <v>199</v>
       </c>
       <c r="E8" t="n">
-        <v>21.2791</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1049</v>
+        <v>0.106</v>
       </c>
       <c r="G8" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="H8" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.0224</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.3958</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.0228</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.3954</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.0229</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.3953</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.0229</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.0423</v>
+      </c>
+      <c r="Q8" t="n">
         <v>0.001</v>
       </c>
-      <c r="H8" t="n">
-        <v>3.51</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.111</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.0406</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.111</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.0407</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.1109</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.0406</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0.0452</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.0045</v>
-      </c>
       <c r="R8" t="n">
-        <v>0.2785</v>
+        <v>0.2707</v>
       </c>
       <c r="S8" t="n">
-        <v>0.0109</v>
+        <v>0.0072</v>
       </c>
       <c r="T8" t="n">
-        <v>0.3306</v>
+        <v>0.317</v>
       </c>
       <c r="U8" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0065</v>
       </c>
       <c r="V8" t="n">
-        <v>9.918200000000001</v>
+        <v>9.509399999999999</v>
       </c>
       <c r="W8" t="n">
-        <v>0.287</v>
+        <v>0.1936</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
@@ -4116,22 +4116,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>47.3548</v>
+        <v>95.8066</v>
       </c>
       <c r="C2" t="n">
-        <v>3.3678</v>
+        <v>12.7824</v>
       </c>
       <c r="D2" t="n">
-        <v>39.2</v>
+        <v>83</v>
       </c>
       <c r="E2" t="n">
-        <v>2.6833</v>
+        <v>11.4018</v>
       </c>
       <c r="F2" t="n">
-        <v>0.035</v>
+        <v>0.037</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0035</v>
+        <v>0.004</v>
       </c>
       <c r="H2" t="n">
         <v>0.68</v>
@@ -4140,46 +4140,46 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8331</v>
+        <v>0.8461</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0113</v>
+        <v>0.0058</v>
       </c>
       <c r="L2" t="n">
-        <v>0.8338</v>
+        <v>0.8467</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0112</v>
+        <v>0.0054</v>
       </c>
       <c r="N2" t="n">
-        <v>0.8313</v>
+        <v>0.84</v>
       </c>
       <c r="O2" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.0064</v>
       </c>
       <c r="P2" t="n">
-        <v>0.1406</v>
+        <v>0.1429</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0017</v>
+        <v>0.0023</v>
       </c>
       <c r="R2" t="n">
-        <v>0.697</v>
+        <v>0.7091</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0101</v>
+        <v>0.0204</v>
       </c>
       <c r="T2" t="n">
-        <v>0.7272</v>
+        <v>0.7389</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0126</v>
+        <v>0.0238</v>
       </c>
       <c r="V2" t="n">
-        <v>8.726699999999999</v>
+        <v>8.8674</v>
       </c>
       <c r="W2" t="n">
-        <v>0.1517</v>
+        <v>0.2861</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -4219,22 +4219,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>64.2683</v>
+        <v>178.1379</v>
       </c>
       <c r="C3" t="n">
-        <v>3.916</v>
+        <v>34.8253</v>
       </c>
       <c r="D3" t="n">
-        <v>39.8</v>
+        <v>118</v>
       </c>
       <c r="E3" t="n">
-        <v>2.3875</v>
+        <v>24.0832</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1521</v>
+        <v>0.1524</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0023</v>
+        <v>0.0017</v>
       </c>
       <c r="H3" t="n">
         <v>2.32</v>
@@ -4243,46 +4243,46 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8316</v>
+        <v>0.861</v>
       </c>
       <c r="K3" t="n">
-        <v>0.016</v>
+        <v>0.013</v>
       </c>
       <c r="L3" t="n">
-        <v>0.8324</v>
+        <v>0.8602</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0151</v>
+        <v>0.0127</v>
       </c>
       <c r="N3" t="n">
-        <v>0.8371</v>
+        <v>0.8597</v>
       </c>
       <c r="O3" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0107</v>
       </c>
       <c r="P3" t="n">
-        <v>0.1691</v>
+        <v>0.1716</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0122</v>
+        <v>0.0102</v>
       </c>
       <c r="R3" t="n">
-        <v>0.7759</v>
+        <v>0.7688</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0306</v>
+        <v>0.0321</v>
       </c>
       <c r="T3" t="n">
-        <v>0.9292</v>
+        <v>0.9314</v>
       </c>
       <c r="U3" t="n">
-        <v>0.0209</v>
+        <v>0.0253</v>
       </c>
       <c r="V3" t="n">
-        <v>11.1501</v>
+        <v>11.1772</v>
       </c>
       <c r="W3" t="n">
-        <v>0.2507</v>
+        <v>0.3042</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -4322,22 +4322,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>61.3298</v>
+        <v>134.312</v>
       </c>
       <c r="C4" t="n">
-        <v>6.2247</v>
+        <v>17.6529</v>
       </c>
       <c r="D4" t="n">
-        <v>41</v>
+        <v>95</v>
       </c>
       <c r="E4" t="n">
-        <v>4.4721</v>
+        <v>12.9422</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1255</v>
+        <v>0.1262</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0007</v>
       </c>
       <c r="H4" t="n">
         <v>1.07</v>
@@ -4346,46 +4346,46 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.8065</v>
+        <v>0.8387</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0205</v>
+        <v>0.0112</v>
       </c>
       <c r="L4" t="n">
-        <v>0.8062</v>
+        <v>0.8388</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0205</v>
+        <v>0.0112</v>
       </c>
       <c r="N4" t="n">
-        <v>0.745</v>
+        <v>0.7514</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0563</v>
+        <v>0.0493</v>
       </c>
       <c r="P4" t="n">
-        <v>0.1582</v>
+        <v>0.1591</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0109</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="R4" t="n">
-        <v>1.2438</v>
+        <v>1.2347</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0477</v>
+        <v>0.0128</v>
       </c>
       <c r="T4" t="n">
-        <v>1.4486</v>
+        <v>1.4847</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0383</v>
+        <v>0.0252</v>
       </c>
       <c r="V4" t="n">
-        <v>17.383</v>
+        <v>17.8165</v>
       </c>
       <c r="W4" t="n">
-        <v>0.4597</v>
+        <v>0.302</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -4425,19 +4425,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>92.7122</v>
+        <v>224.7787</v>
       </c>
       <c r="C5" t="n">
-        <v>10.8141</v>
+        <v>50.5633</v>
       </c>
       <c r="D5" t="n">
-        <v>43</v>
+        <v>110</v>
       </c>
       <c r="E5" t="n">
-        <v>5.4772</v>
+        <v>25.836</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3156</v>
+        <v>0.316</v>
       </c>
       <c r="G5" t="n">
         <v>0.0022</v>
@@ -4449,46 +4449,46 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8608</v>
+        <v>0.8753</v>
       </c>
       <c r="K5" t="n">
-        <v>0.013</v>
+        <v>0.0129</v>
       </c>
       <c r="L5" t="n">
-        <v>0.8599</v>
+        <v>0.875</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0133</v>
+        <v>0.0122</v>
       </c>
       <c r="N5" t="n">
-        <v>0.6912</v>
+        <v>0.6812</v>
       </c>
       <c r="O5" t="n">
-        <v>0.0277</v>
+        <v>0.0822</v>
       </c>
       <c r="P5" t="n">
-        <v>0.2452</v>
+        <v>0.2437</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.0041</v>
+        <v>0.0137</v>
       </c>
       <c r="R5" t="n">
-        <v>0.9916</v>
+        <v>1.0027</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0191</v>
+        <v>0.0228</v>
       </c>
       <c r="T5" t="n">
-        <v>1.5693</v>
+        <v>1.5888</v>
       </c>
       <c r="U5" t="n">
-        <v>0.012</v>
+        <v>0.0187</v>
       </c>
       <c r="V5" t="n">
-        <v>18.8311</v>
+        <v>19.0653</v>
       </c>
       <c r="W5" t="n">
-        <v>0.144</v>
+        <v>0.2243</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -4528,22 +4528,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>84.7109</v>
+        <v>312.4196</v>
       </c>
       <c r="C6" t="n">
-        <v>24.5372</v>
+        <v>39.4625</v>
       </c>
       <c r="D6" t="n">
-        <v>46.4</v>
+        <v>182</v>
       </c>
       <c r="E6" t="n">
-        <v>13.5019</v>
+        <v>23.3452</v>
       </c>
       <c r="F6" t="n">
         <v>0.1829</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0003</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="H6" t="n">
         <v>7.13</v>
@@ -4552,46 +4552,46 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.6923</v>
+        <v>0.8768</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0746</v>
+        <v>0.0156</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6912</v>
+        <v>0.877</v>
       </c>
       <c r="M6" t="n">
-        <v>0.07489999999999999</v>
+        <v>0.0159</v>
       </c>
       <c r="N6" t="n">
-        <v>0.5981</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0983</v>
+        <v>0.0226</v>
       </c>
       <c r="P6" t="n">
-        <v>0.205</v>
+        <v>0.2044</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0074</v>
       </c>
       <c r="R6" t="n">
-        <v>0.7593</v>
+        <v>0.7873</v>
       </c>
       <c r="S6" t="n">
-        <v>0.0124</v>
+        <v>0.0175</v>
       </c>
       <c r="T6" t="n">
-        <v>0.9469</v>
+        <v>0.9617</v>
       </c>
       <c r="U6" t="n">
-        <v>0.0145</v>
+        <v>0.048</v>
       </c>
       <c r="V6" t="n">
-        <v>11.3627</v>
+        <v>11.5406</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1737</v>
+        <v>0.5764</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -4631,19 +4631,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>58.9315</v>
+        <v>277.6454</v>
       </c>
       <c r="C7" t="n">
-        <v>1.7498</v>
+        <v>1.0524</v>
       </c>
       <c r="D7" t="n">
-        <v>38.8</v>
+        <v>199</v>
       </c>
       <c r="E7" t="n">
-        <v>0.4472</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1114</v>
+        <v>0.1119</v>
       </c>
       <c r="G7" t="n">
         <v>0.0005</v>
@@ -4655,46 +4655,46 @@
         <v>0.0055</v>
       </c>
       <c r="J7" t="n">
-        <v>0.7195</v>
+        <v>0.878</v>
       </c>
       <c r="K7" t="n">
-        <v>0.027</v>
+        <v>0.0067</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7181999999999999</v>
+        <v>0.8782</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0272</v>
+        <v>0.0067</v>
       </c>
       <c r="N7" t="n">
-        <v>0.7062</v>
+        <v>0.8763</v>
       </c>
       <c r="O7" t="n">
-        <v>0.029</v>
+        <v>0.0083</v>
       </c>
       <c r="P7" t="n">
-        <v>0.1779</v>
+        <v>0.1495</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0062</v>
+        <v>0.0043</v>
       </c>
       <c r="R7" t="n">
-        <v>0.6599</v>
+        <v>0.6919</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0115</v>
+        <v>0.0282</v>
       </c>
       <c r="T7" t="n">
-        <v>0.7392</v>
+        <v>0.7472</v>
       </c>
       <c r="U7" t="n">
-        <v>0.0145</v>
+        <v>0.0136</v>
       </c>
       <c r="V7" t="n">
-        <v>8.8706</v>
+        <v>8.966100000000001</v>
       </c>
       <c r="W7" t="n">
-        <v>0.1743</v>
+        <v>0.163</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -4734,70 +4734,70 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>55.3798</v>
+        <v>262.8867</v>
       </c>
       <c r="C8" t="n">
-        <v>1.123</v>
+        <v>3.5415</v>
       </c>
       <c r="D8" t="n">
-        <v>38.8</v>
+        <v>199</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4472</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1015</v>
+        <v>0.1031</v>
       </c>
       <c r="G8" t="n">
-        <v>0.001</v>
+        <v>0.0008</v>
       </c>
       <c r="H8" t="n">
-        <v>2.81</v>
+        <v>2.814</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>0.0089</v>
       </c>
       <c r="J8" t="n">
-        <v>0.7058</v>
+        <v>0.8696</v>
       </c>
       <c r="K8" t="n">
-        <v>0.021</v>
+        <v>0.0073</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7054</v>
+        <v>0.8702</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0214</v>
+        <v>0.0073</v>
       </c>
       <c r="N8" t="n">
-        <v>0.6916</v>
+        <v>0.8696</v>
       </c>
       <c r="O8" t="n">
-        <v>0.0355</v>
+        <v>0.0068</v>
       </c>
       <c r="P8" t="n">
-        <v>0.1468</v>
+        <v>0.1392</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.0105</v>
+        <v>0.0034</v>
       </c>
       <c r="R8" t="n">
-        <v>0.7004</v>
+        <v>0.6622</v>
       </c>
       <c r="S8" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0067</v>
       </c>
       <c r="T8" t="n">
-        <v>0.8046</v>
+        <v>0.7863</v>
       </c>
       <c r="U8" t="n">
-        <v>0.0217</v>
+        <v>0.0148</v>
       </c>
       <c r="V8" t="n">
-        <v>9.655099999999999</v>
+        <v>9.4353</v>
       </c>
       <c r="W8" t="n">
-        <v>0.2603</v>
+        <v>0.1777</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
@@ -4998,70 +4998,70 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>34.5481</v>
+        <v>42.9973</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9897</v>
+        <v>3.1193</v>
       </c>
       <c r="D2" t="n">
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="E2" t="n">
-        <v>4.4721</v>
+        <v>10.8397</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0295</v>
+        <v>0.0297</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0003</v>
+        <v>0.0004</v>
       </c>
       <c r="H2" t="n">
-        <v>0.768</v>
+        <v>0.8</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0622</v>
+        <v>0.0308</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6473</v>
+        <v>0.6543</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0132</v>
+        <v>0.0151</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6477000000000001</v>
+        <v>0.6543</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0141</v>
+        <v>0.0144</v>
       </c>
       <c r="N2" t="n">
-        <v>0.6363</v>
+        <v>0.6474</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0194</v>
+        <v>0.0168</v>
       </c>
       <c r="P2" t="n">
-        <v>0.1662</v>
+        <v>0.1691</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0028</v>
+        <v>0.0045</v>
       </c>
       <c r="R2" t="n">
-        <v>0.4033</v>
+        <v>0.4008</v>
       </c>
       <c r="S2" t="n">
-        <v>0.005</v>
+        <v>0.0041</v>
       </c>
       <c r="T2" t="n">
-        <v>0.509</v>
+        <v>0.5096000000000001</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0021</v>
+        <v>0.0055</v>
       </c>
       <c r="V2" t="n">
-        <v>3.0537</v>
+        <v>3.0574</v>
       </c>
       <c r="W2" t="n">
-        <v>0.0127</v>
+        <v>0.033</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -5101,70 +5101,70 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>51.6329</v>
+        <v>63.6435</v>
       </c>
       <c r="C3" t="n">
-        <v>2.3252</v>
+        <v>6.3142</v>
       </c>
       <c r="D3" t="n">
-        <v>109</v>
+        <v>139</v>
       </c>
       <c r="E3" t="n">
-        <v>6.1237</v>
+        <v>15.8114</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1573</v>
+        <v>0.157</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0015</v>
+        <v>0.0016</v>
       </c>
       <c r="H3" t="n">
-        <v>1.864</v>
+        <v>1.872</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0537</v>
+        <v>0.0179</v>
       </c>
       <c r="J3" t="n">
-        <v>0.7454</v>
+        <v>0.7521</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0256</v>
+        <v>0.0139</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7486</v>
+        <v>0.7562</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0257</v>
+        <v>0.0111</v>
       </c>
       <c r="N3" t="n">
-        <v>0.7379</v>
+        <v>0.7456</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0216</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="P3" t="n">
-        <v>0.2221</v>
+        <v>0.227</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0221</v>
+        <v>0.0246</v>
       </c>
       <c r="R3" t="n">
-        <v>0.504</v>
+        <v>0.509</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0252</v>
+        <v>0.0294</v>
       </c>
       <c r="T3" t="n">
-        <v>0.8585</v>
+        <v>0.8697</v>
       </c>
       <c r="U3" t="n">
-        <v>0.0332</v>
+        <v>0.0365</v>
       </c>
       <c r="V3" t="n">
-        <v>5.1512</v>
+        <v>5.218</v>
       </c>
       <c r="W3" t="n">
-        <v>0.1992</v>
+        <v>0.2193</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -5204,70 +5204,70 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>46.0636</v>
+        <v>63.0023</v>
       </c>
       <c r="C4" t="n">
-        <v>2.4588</v>
+        <v>4.6552</v>
       </c>
       <c r="D4" t="n">
-        <v>111</v>
+        <v>155</v>
       </c>
       <c r="E4" t="n">
-        <v>5.7009</v>
+        <v>11.9373</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1303</v>
+        <v>0.1301</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0022</v>
+        <v>0.0017</v>
       </c>
       <c r="H4" t="n">
-        <v>0.862</v>
+        <v>0.896</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0179</v>
+        <v>0.0195</v>
       </c>
       <c r="J4" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.7078</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0439</v>
+        <v>0.0241</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6859</v>
+        <v>0.7115</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0447</v>
+        <v>0.0258</v>
       </c>
       <c r="N4" t="n">
-        <v>0.6525</v>
+        <v>0.6208</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0489</v>
+        <v>0.0357</v>
       </c>
       <c r="P4" t="n">
-        <v>0.2226</v>
+        <v>0.1935</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0273</v>
+        <v>0.0233</v>
       </c>
       <c r="R4" t="n">
-        <v>0.492</v>
+        <v>0.5131</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0036</v>
+        <v>0.0275</v>
       </c>
       <c r="T4" t="n">
-        <v>1.105</v>
+        <v>1.1232</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0359</v>
+        <v>0.0362</v>
       </c>
       <c r="V4" t="n">
-        <v>6.6298</v>
+        <v>6.739</v>
       </c>
       <c r="W4" t="n">
-        <v>0.2153</v>
+        <v>0.2169</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -5307,70 +5307,70 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>75.09399999999999</v>
+        <v>107.8128</v>
       </c>
       <c r="C5" t="n">
-        <v>2.8956</v>
+        <v>21.9706</v>
       </c>
       <c r="D5" t="n">
-        <v>110</v>
+        <v>162</v>
       </c>
       <c r="E5" t="n">
-        <v>4.1833</v>
+        <v>34.2053</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2952</v>
+        <v>0.2965</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0014</v>
+        <v>0.002</v>
       </c>
       <c r="H5" t="n">
-        <v>6.448</v>
+        <v>6.456</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0179</v>
+        <v>0.0219</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7035</v>
+        <v>0.6977</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0429</v>
+        <v>0.0365</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7052</v>
+        <v>0.6982</v>
       </c>
       <c r="M5" t="n">
-        <v>0.043</v>
+        <v>0.0386</v>
       </c>
       <c r="N5" t="n">
-        <v>0.5599</v>
+        <v>0.5525</v>
       </c>
       <c r="O5" t="n">
-        <v>0.1397</v>
+        <v>0.1179</v>
       </c>
       <c r="P5" t="n">
-        <v>0.3623</v>
+        <v>0.3561</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.0034</v>
+        <v>0.0263</v>
       </c>
       <c r="R5" t="n">
-        <v>0.916</v>
+        <v>0.8987000000000001</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0419</v>
+        <v>0.0223</v>
       </c>
       <c r="T5" t="n">
-        <v>2.211</v>
+        <v>2.2064</v>
       </c>
       <c r="U5" t="n">
-        <v>0.0273</v>
+        <v>0.0259</v>
       </c>
       <c r="V5" t="n">
-        <v>13.2662</v>
+        <v>13.2386</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1639</v>
+        <v>0.1554</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -5410,70 +5410,70 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64.6746</v>
+        <v>77.9144</v>
       </c>
       <c r="C6" t="n">
-        <v>2.5369</v>
+        <v>4.9424</v>
       </c>
       <c r="D6" t="n">
-        <v>106</v>
+        <v>133</v>
       </c>
       <c r="E6" t="n">
-        <v>4.4721</v>
+        <v>8.9443</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1636</v>
+        <v>0.1643</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0003</v>
+        <v>0.0014</v>
       </c>
       <c r="H6" t="n">
-        <v>5.736</v>
+        <v>5.79</v>
       </c>
       <c r="I6" t="n">
-        <v>0.065</v>
+        <v>0.0424</v>
       </c>
       <c r="J6" t="n">
-        <v>0.6042</v>
+        <v>0.6045</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0027</v>
+        <v>0.0051</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6048</v>
+        <v>0.6046</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0018</v>
+        <v>0.0045</v>
       </c>
       <c r="N6" t="n">
-        <v>0.5894</v>
+        <v>0.5896</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0095</v>
+        <v>0.0141</v>
       </c>
       <c r="P6" t="n">
-        <v>0.2765</v>
+        <v>0.2783</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.0058</v>
+        <v>0.0205</v>
       </c>
       <c r="R6" t="n">
-        <v>0.5245</v>
+        <v>0.5132</v>
       </c>
       <c r="S6" t="n">
-        <v>0.0245</v>
+        <v>0.006</v>
       </c>
       <c r="T6" t="n">
-        <v>1.0278</v>
+        <v>1.0028</v>
       </c>
       <c r="U6" t="n">
-        <v>0.0354</v>
+        <v>0.0273</v>
       </c>
       <c r="V6" t="n">
-        <v>6.1668</v>
+        <v>6.0171</v>
       </c>
       <c r="W6" t="n">
-        <v>0.2123</v>
+        <v>0.1637</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -5513,70 +5513,70 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>48.6507</v>
+        <v>56.2247</v>
       </c>
       <c r="C7" t="n">
-        <v>3.4735</v>
+        <v>5.0812</v>
       </c>
       <c r="D7" t="n">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="E7" t="n">
-        <v>8.660299999999999</v>
+        <v>13.0384</v>
       </c>
       <c r="F7" t="n">
-        <v>0.104</v>
+        <v>0.1044</v>
       </c>
       <c r="G7" t="n">
-        <v>0.001</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>3.412</v>
+        <v>3.48</v>
       </c>
       <c r="I7" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.1562</v>
       </c>
       <c r="J7" t="n">
-        <v>0.6052</v>
+        <v>0.613</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0074</v>
+        <v>0.0046</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6046</v>
+        <v>0.6131</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0071</v>
+        <v>0.0044</v>
       </c>
       <c r="N7" t="n">
-        <v>0.5503</v>
+        <v>0.577</v>
       </c>
       <c r="O7" t="n">
-        <v>0.1222</v>
+        <v>0.0379</v>
       </c>
       <c r="P7" t="n">
-        <v>0.1826</v>
+        <v>0.187</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0056</v>
+        <v>0.0064</v>
       </c>
       <c r="R7" t="n">
-        <v>0.3664</v>
+        <v>0.3535</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0354</v>
+        <v>0.0214</v>
       </c>
       <c r="T7" t="n">
-        <v>0.5762</v>
+        <v>0.5827</v>
       </c>
       <c r="U7" t="n">
-        <v>0.0047</v>
+        <v>0.0081</v>
       </c>
       <c r="V7" t="n">
-        <v>3.4575</v>
+        <v>3.496</v>
       </c>
       <c r="W7" t="n">
-        <v>0.0279</v>
+        <v>0.0489</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -5616,70 +5616,70 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>44.7079</v>
+        <v>51.4643</v>
       </c>
       <c r="C8" t="n">
-        <v>2.7248</v>
+        <v>3.3934</v>
       </c>
       <c r="D8" t="n">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="E8" t="n">
-        <v>8.3666</v>
+        <v>10.9545</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1048</v>
+        <v>0.1055</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0007</v>
+        <v>0.0016</v>
       </c>
       <c r="H8" t="n">
-        <v>2.256</v>
+        <v>2.416</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1048</v>
+        <v>0.4454</v>
       </c>
       <c r="J8" t="n">
-        <v>0.6125</v>
+        <v>0.6074000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0053</v>
+        <v>0.0046</v>
       </c>
       <c r="L8" t="n">
-        <v>0.6127</v>
+        <v>0.608</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0069</v>
+        <v>0.0047</v>
       </c>
       <c r="N8" t="n">
-        <v>0.6104000000000001</v>
+        <v>0.6092</v>
       </c>
       <c r="O8" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.0059</v>
       </c>
       <c r="P8" t="n">
-        <v>0.164</v>
+        <v>0.1649</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.0037</v>
+        <v>0.0027</v>
       </c>
       <c r="R8" t="n">
-        <v>0.349</v>
+        <v>0.3365</v>
       </c>
       <c r="S8" t="n">
+        <v>0.0042</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.6385999999999999</v>
+      </c>
+      <c r="U8" t="n">
         <v>0.0236</v>
       </c>
-      <c r="T8" t="n">
-        <v>0.6497000000000001</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0.0339</v>
-      </c>
       <c r="V8" t="n">
-        <v>3.8979</v>
+        <v>3.8314</v>
       </c>
       <c r="W8" t="n">
-        <v>0.2032</v>
+        <v>0.1419</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
@@ -5880,70 +5880,70 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>37.1667</v>
+        <v>48.1218</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5542</v>
+        <v>4.8378</v>
       </c>
       <c r="D2" t="n">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="E2" t="n">
-        <v>2.7386</v>
+        <v>16.0468</v>
       </c>
       <c r="F2" t="n">
         <v>0.0307</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0002</v>
+        <v>0.0004</v>
       </c>
       <c r="H2" t="n">
-        <v>0.786</v>
+        <v>0.762</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0219</v>
+        <v>0.0963</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6477000000000001</v>
+        <v>0.6605</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0112</v>
+        <v>0.0125</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5951</v>
+        <v>0.6091</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0139</v>
+        <v>0.0152</v>
       </c>
       <c r="N2" t="n">
-        <v>0.6092</v>
+        <v>0.6198</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0135</v>
+        <v>0.0133</v>
       </c>
       <c r="P2" t="n">
-        <v>0.1935</v>
+        <v>0.1946</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0055</v>
+        <v>0.0038</v>
       </c>
       <c r="R2" t="n">
-        <v>0.5492</v>
+        <v>0.5562</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0146</v>
+        <v>0.0041</v>
       </c>
       <c r="T2" t="n">
-        <v>0.6689000000000001</v>
+        <v>0.6625</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0108</v>
+        <v>0.0136</v>
       </c>
       <c r="V2" t="n">
-        <v>4.0133</v>
+        <v>3.9748</v>
       </c>
       <c r="W2" t="n">
-        <v>0.06510000000000001</v>
+        <v>0.0818</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -5983,70 +5983,70 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>54.8965</v>
+        <v>69.98739999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>2.7968</v>
+        <v>8.258599999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>110</v>
+        <v>143</v>
       </c>
       <c r="E3" t="n">
-        <v>5.4772</v>
+        <v>17.4642</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1585</v>
+        <v>0.1582</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0029</v>
+        <v>0.0014</v>
       </c>
       <c r="H3" t="n">
-        <v>1.876</v>
+        <v>1.838</v>
       </c>
       <c r="I3" t="n">
-        <v>0.07770000000000001</v>
+        <v>0.0383</v>
       </c>
       <c r="J3" t="n">
-        <v>0.643</v>
+        <v>0.6705</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0234</v>
+        <v>0.0178</v>
       </c>
       <c r="L3" t="n">
-        <v>0.5833</v>
+        <v>0.616</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0188</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="N3" t="n">
-        <v>0.5893</v>
+        <v>0.5999</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0222</v>
+        <v>0.0246</v>
       </c>
       <c r="P3" t="n">
-        <v>0.2554</v>
+        <v>0.2511</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0268</v>
+        <v>0.0278</v>
       </c>
       <c r="R3" t="n">
-        <v>0.6636</v>
+        <v>0.6652</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0271</v>
+        <v>0.0319</v>
       </c>
       <c r="T3" t="n">
-        <v>0.9852</v>
+        <v>1.0249</v>
       </c>
       <c r="U3" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0351</v>
       </c>
       <c r="V3" t="n">
-        <v>5.9114</v>
+        <v>6.1495</v>
       </c>
       <c r="W3" t="n">
-        <v>0.049</v>
+        <v>0.2109</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -6086,70 +6086,70 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>49.7985</v>
+        <v>72.14490000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>1.3219</v>
+        <v>11.0091</v>
       </c>
       <c r="D4" t="n">
-        <v>113</v>
+        <v>168</v>
       </c>
       <c r="E4" t="n">
-        <v>4.1833</v>
+        <v>27.2489</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1315</v>
+        <v>0.1297</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0011</v>
+        <v>0.001</v>
       </c>
       <c r="H4" t="n">
-        <v>0.874</v>
+        <v>0.886</v>
       </c>
       <c r="I4" t="n">
-        <v>0.055</v>
+        <v>0.0434</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.6067</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0541</v>
+        <v>0.0409</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4865</v>
+        <v>0.539</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0585</v>
+        <v>0.0587</v>
       </c>
       <c r="N4" t="n">
-        <v>0.3961</v>
+        <v>0.4197</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0187</v>
+        <v>0.0291</v>
       </c>
       <c r="P4" t="n">
-        <v>0.2203</v>
+        <v>0.202</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0284</v>
+        <v>0.0027</v>
       </c>
       <c r="R4" t="n">
-        <v>0.8308</v>
+        <v>0.8106</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0307</v>
+        <v>0.0257</v>
       </c>
       <c r="T4" t="n">
-        <v>1.3844</v>
+        <v>1.3579</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0118</v>
+        <v>0.0131</v>
       </c>
       <c r="V4" t="n">
-        <v>8.3066</v>
+        <v>8.147500000000001</v>
       </c>
       <c r="W4" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.07870000000000001</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -6189,70 +6189,70 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>77.0663</v>
+        <v>118.1362</v>
       </c>
       <c r="C5" t="n">
-        <v>4.087</v>
+        <v>16.3217</v>
       </c>
       <c r="D5" t="n">
-        <v>110</v>
+        <v>170</v>
       </c>
       <c r="E5" t="n">
-        <v>4.1833</v>
+        <v>24.3413</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2974</v>
+        <v>0.2983</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0018</v>
+        <v>0.0015</v>
       </c>
       <c r="H5" t="n">
-        <v>6.456</v>
+        <v>6.488</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0219</v>
+        <v>0.0179</v>
       </c>
       <c r="J5" t="n">
-        <v>0.6011</v>
+        <v>0.6368</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0147</v>
+        <v>0.0192</v>
       </c>
       <c r="L5" t="n">
-        <v>0.5246</v>
+        <v>0.5558</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0244</v>
+        <v>0.0449</v>
       </c>
       <c r="N5" t="n">
-        <v>0.3257</v>
+        <v>0.3435</v>
       </c>
       <c r="O5" t="n">
-        <v>0.0121</v>
+        <v>0.0253</v>
       </c>
       <c r="P5" t="n">
-        <v>0.3543</v>
+        <v>0.3917</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.031</v>
+        <v>0.0059</v>
       </c>
       <c r="R5" t="n">
-        <v>1.1077</v>
+        <v>1.0683</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0152</v>
+        <v>0.0248</v>
       </c>
       <c r="T5" t="n">
-        <v>2.3701</v>
+        <v>2.3457</v>
       </c>
       <c r="U5" t="n">
-        <v>0.0325</v>
+        <v>0.0373</v>
       </c>
       <c r="V5" t="n">
-        <v>14.2206</v>
+        <v>14.0742</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1951</v>
+        <v>0.2238</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -6292,70 +6292,70 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>86.33320000000001</v>
+        <v>135.7699</v>
       </c>
       <c r="C6" t="n">
-        <v>14.1691</v>
+        <v>2.0528</v>
       </c>
       <c r="D6" t="n">
-        <v>124</v>
+        <v>199</v>
       </c>
       <c r="E6" t="n">
-        <v>19.3649</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>0.1655</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0011</v>
+        <v>0.0008</v>
       </c>
       <c r="H6" t="n">
-        <v>5.732</v>
+        <v>5.778</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0045</v>
+        <v>0.06909999999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4962</v>
+        <v>0.63</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0658</v>
+        <v>0.037</v>
       </c>
       <c r="L6" t="n">
-        <v>0.4749</v>
+        <v>0.6048</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0575</v>
+        <v>0.034</v>
       </c>
       <c r="N6" t="n">
-        <v>0.4443</v>
+        <v>0.5725</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0546</v>
+        <v>0.0171</v>
       </c>
       <c r="P6" t="n">
-        <v>0.3142</v>
+        <v>0.2972</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.0266</v>
+        <v>0.0058</v>
       </c>
       <c r="R6" t="n">
-        <v>0.6629</v>
+        <v>0.6653</v>
       </c>
       <c r="S6" t="n">
-        <v>0.0111</v>
+        <v>0.0055</v>
       </c>
       <c r="T6" t="n">
-        <v>1.1522</v>
+        <v>1.1411</v>
       </c>
       <c r="U6" t="n">
-        <v>0.0269</v>
+        <v>0.0092</v>
       </c>
       <c r="V6" t="n">
-        <v>6.9134</v>
+        <v>6.8468</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1616</v>
+        <v>0.0549</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -6395,70 +6395,70 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>61.8054</v>
+        <v>96.6665</v>
       </c>
       <c r="C7" t="n">
-        <v>8.3467</v>
+        <v>1.3598</v>
       </c>
       <c r="D7" t="n">
-        <v>125</v>
+        <v>199</v>
       </c>
       <c r="E7" t="n">
-        <v>17.1026</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1049</v>
+        <v>0.1046</v>
       </c>
       <c r="G7" t="n">
-        <v>0.001</v>
+        <v>0.0005</v>
       </c>
       <c r="H7" t="n">
         <v>3.398</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0955</v>
+        <v>0.0517</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4998</v>
+        <v>0.5972</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0598</v>
+        <v>0.0196</v>
       </c>
       <c r="L7" t="n">
-        <v>0.4795</v>
+        <v>0.5631</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0498</v>
+        <v>0.0195</v>
       </c>
       <c r="N7" t="n">
-        <v>0.4555</v>
+        <v>0.555</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0444</v>
+        <v>0.0156</v>
       </c>
       <c r="P7" t="n">
-        <v>0.2062</v>
+        <v>0.2112</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0041</v>
+        <v>0.0033</v>
       </c>
       <c r="R7" t="n">
-        <v>0.4984</v>
+        <v>0.4985</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0275</v>
+        <v>0.0056</v>
       </c>
       <c r="T7" t="n">
-        <v>0.731</v>
+        <v>0.7391</v>
       </c>
       <c r="U7" t="n">
-        <v>0.0056</v>
+        <v>0.0111</v>
       </c>
       <c r="V7" t="n">
-        <v>4.3858</v>
+        <v>4.4344</v>
       </c>
       <c r="W7" t="n">
-        <v>0.0337</v>
+        <v>0.0664</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -6498,70 +6498,70 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50.2461</v>
+        <v>79.1786</v>
       </c>
       <c r="C8" t="n">
-        <v>11.987</v>
+        <v>2.2669</v>
       </c>
       <c r="D8" t="n">
-        <v>122</v>
+        <v>197</v>
       </c>
       <c r="E8" t="n">
-        <v>29.2831</v>
+        <v>4.4721</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1046</v>
+        <v>0.105</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0011</v>
       </c>
       <c r="H8" t="n">
-        <v>2.242</v>
+        <v>2.342</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0438</v>
+        <v>0.1564</v>
       </c>
       <c r="J8" t="n">
-        <v>0.4517</v>
+        <v>0.5599</v>
       </c>
       <c r="K8" t="n">
-        <v>0.1063</v>
+        <v>0.0181</v>
       </c>
       <c r="L8" t="n">
-        <v>0.4076</v>
+        <v>0.5037</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0987</v>
+        <v>0.0206</v>
       </c>
       <c r="N8" t="n">
-        <v>0.3974</v>
+        <v>0.4792</v>
       </c>
       <c r="O8" t="n">
-        <v>0.0771</v>
+        <v>0.0364</v>
       </c>
       <c r="P8" t="n">
-        <v>0.1812</v>
+        <v>0.1835</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.003</v>
+        <v>0.0062</v>
       </c>
       <c r="R8" t="n">
-        <v>0.5088</v>
+        <v>0.5067</v>
       </c>
       <c r="S8" t="n">
-        <v>0.0101</v>
+        <v>0.0229</v>
       </c>
       <c r="T8" t="n">
-        <v>0.7991</v>
+        <v>0.8072</v>
       </c>
       <c r="U8" t="n">
-        <v>0.0381</v>
+        <v>0.0254</v>
       </c>
       <c r="V8" t="n">
-        <v>4.7943</v>
+        <v>4.8431</v>
       </c>
       <c r="W8" t="n">
-        <v>0.2288</v>
+        <v>0.1525</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>

</xml_diff>